<commit_message>
Removed Empty Rows for BOM
</commit_message>
<xml_diff>
--- a/resources/v0.1.2/design_documents/BOM-V0.1.2.xlsx
+++ b/resources/v0.1.2/design_documents/BOM-V0.1.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ig2\Desktop\SMR Thermal\thermal-loop\resources\v0.1.2\design_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0CC7EB-E376-4619-9A43-94EBDD984420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8EFCAD-E538-49A4-B1BC-B069F4E5ED81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -1333,8 +1333,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K122" totalsRowShown="0" tableBorderDxfId="7">
-  <autoFilter ref="A1:K122" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K116" totalsRowShown="0" tableBorderDxfId="7">
+  <autoFilter ref="A1:K116" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{7B25C464-EB0A-4B56-94DE-96F6AA8DEAC1}" name="Internal Part Name" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{DF8C1AF7-50DF-4DF9-864F-041981FCACF8}" name="MFR / Vendor Description" dataDxfId="5"/>
@@ -1671,7 +1671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:M122"/>
+  <dimension ref="A1:M116"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
@@ -3349,7 +3349,7 @@
         <v>45.81</v>
       </c>
       <c r="F67" s="6">
-        <f t="shared" ref="F67:F109" si="1">D67*E67</f>
+        <f t="shared" ref="F67:F103" si="1">D67*E67</f>
         <v>45.81</v>
       </c>
       <c r="H67" s="23" t="s">
@@ -3971,7 +3971,7 @@
         <v>110</v>
       </c>
       <c r="F93" s="6">
-        <f t="shared" ref="F93:F101" si="2">D93*E93</f>
+        <f t="shared" ref="F93:F95" si="2">D93*E93</f>
         <v>110</v>
       </c>
       <c r="H93" s="24" t="s">
@@ -4027,519 +4027,447 @@
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A96" s="13"/>
+      <c r="A96" s="14" t="s">
+        <v>68</v>
+      </c>
       <c r="B96" s="26"/>
-      <c r="C96" s="13"/>
-      <c r="D96" s="7"/>
-      <c r="E96" s="7"/>
+      <c r="C96" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="D96" s="8">
+        <v>3</v>
+      </c>
+      <c r="E96" s="8">
+        <v>2.1800000000000002</v>
+      </c>
       <c r="F96" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H96" s="24"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A97" s="13"/>
+        <f t="shared" si="1"/>
+        <v>6.5400000000000009</v>
+      </c>
+      <c r="H96" s="25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A97" s="13" t="s">
+        <v>69</v>
+      </c>
       <c r="B97" s="26"/>
-      <c r="C97" s="13"/>
-      <c r="D97" s="7"/>
-      <c r="E97" s="7"/>
+      <c r="C97" s="13">
+        <v>156665159304</v>
+      </c>
+      <c r="D97" s="7">
+        <v>3</v>
+      </c>
+      <c r="E97" s="7">
+        <v>35.97</v>
+      </c>
       <c r="F97" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H97" s="24"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A98" s="13"/>
-      <c r="B98" s="26"/>
-      <c r="C98" s="13"/>
-      <c r="D98" s="7"/>
-      <c r="E98" s="7"/>
+        <f t="shared" si="1"/>
+        <v>107.91</v>
+      </c>
+      <c r="H97" s="24" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A98" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B98" s="26" t="s">
+        <v>240</v>
+      </c>
+      <c r="C98" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="D98" s="8">
+        <v>3</v>
+      </c>
+      <c r="E98" s="8">
+        <v>167.42</v>
+      </c>
       <c r="F98" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H98" s="24"/>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A99" s="13"/>
-      <c r="B99" s="26"/>
-      <c r="C99" s="13"/>
-      <c r="D99" s="7"/>
-      <c r="E99" s="7"/>
+        <f t="shared" si="1"/>
+        <v>502.26</v>
+      </c>
+      <c r="H98" s="23" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A99" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B99" s="26" t="s">
+        <v>249</v>
+      </c>
+      <c r="C99" s="13">
+        <v>316529</v>
+      </c>
+      <c r="D99" s="7">
+        <v>1</v>
+      </c>
+      <c r="E99" s="7">
+        <v>405</v>
+      </c>
       <c r="F99" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H99" s="24"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A100" s="13"/>
-      <c r="B100" s="26"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="7"/>
-      <c r="E100" s="7"/>
+        <f t="shared" si="1"/>
+        <v>405</v>
+      </c>
+      <c r="H99" s="22" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A100" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B100" s="26" t="s">
+        <v>250</v>
+      </c>
+      <c r="C100" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D100" s="8">
+        <v>1</v>
+      </c>
+      <c r="E100" s="8">
+        <v>37.4</v>
+      </c>
       <c r="F100" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H100" s="24"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A101" s="13"/>
-      <c r="B101" s="26"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="7"/>
-      <c r="E101" s="7"/>
+        <f t="shared" si="1"/>
+        <v>37.4</v>
+      </c>
+      <c r="H100" s="23" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A101" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B101" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C101" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D101" s="7">
+        <v>1</v>
+      </c>
+      <c r="E101" s="7">
+        <v>20.91</v>
+      </c>
       <c r="F101" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H101" s="24"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>20.91</v>
+      </c>
+      <c r="H101" s="22" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B102" s="26"/>
-      <c r="C102" s="14" t="s">
-        <v>150</v>
+        <v>61</v>
+      </c>
+      <c r="B102" s="26" t="s">
+        <v>251</v>
+      </c>
+      <c r="C102" s="11" t="s">
+        <v>74</v>
       </c>
       <c r="D102" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E102" s="8">
-        <v>2.1800000000000002</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="F102" s="6">
         <f t="shared" si="1"/>
-        <v>6.5400000000000009</v>
-      </c>
-      <c r="H102" s="25" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="H102" s="23" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="B103" s="26"/>
-      <c r="C103" s="13">
-        <v>156665159304</v>
+        <v>71</v>
+      </c>
+      <c r="B103" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="C103" s="17" t="s">
+        <v>153</v>
       </c>
       <c r="D103" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E103" s="7">
-        <v>35.97</v>
+        <v>16.260000000000002</v>
       </c>
       <c r="F103" s="6">
         <f t="shared" si="1"/>
-        <v>107.91</v>
-      </c>
-      <c r="H103" s="24" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A104" s="14" t="s">
-        <v>67</v>
+        <v>16.260000000000002</v>
+      </c>
+      <c r="H103" s="22" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A104" s="27" t="s">
+        <v>258</v>
       </c>
       <c r="B104" s="26" t="s">
-        <v>240</v>
-      </c>
-      <c r="C104" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="D104" s="8">
-        <v>3</v>
-      </c>
-      <c r="E104" s="8">
-        <v>167.42</v>
+        <v>254</v>
+      </c>
+      <c r="C104" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="D104" s="28">
+        <v>1</v>
+      </c>
+      <c r="E104" s="28">
+        <v>5.35</v>
       </c>
       <c r="F104" s="6">
-        <f t="shared" si="1"/>
-        <v>502.26</v>
-      </c>
-      <c r="H104" s="23" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A105" s="13" t="s">
-        <v>70</v>
+        <f>D104*E104</f>
+        <v>5.35</v>
+      </c>
+      <c r="H104" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A105" s="27" t="s">
+        <v>259</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>249</v>
-      </c>
-      <c r="C105" s="13">
-        <v>316529</v>
-      </c>
-      <c r="D105" s="7">
-        <v>1</v>
-      </c>
-      <c r="E105" s="7">
-        <v>405</v>
+        <v>256</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="D105" s="28">
+        <v>1</v>
+      </c>
+      <c r="E105" s="28">
+        <v>10.75</v>
       </c>
       <c r="F105" s="6">
-        <f t="shared" si="1"/>
-        <v>405</v>
-      </c>
-      <c r="H105" s="22" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A106" s="14" t="s">
-        <v>66</v>
+        <f>D105*E105</f>
+        <v>10.75</v>
+      </c>
+      <c r="H105" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A106" s="27" t="s">
+        <v>260</v>
       </c>
       <c r="B106" s="26" t="s">
-        <v>250</v>
-      </c>
-      <c r="C106" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="D106" s="8">
-        <v>1</v>
-      </c>
-      <c r="E106" s="8">
-        <v>37.4</v>
+        <v>263</v>
+      </c>
+      <c r="C106" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="D106" s="28">
+        <v>1</v>
+      </c>
+      <c r="E106" s="28">
+        <v>6.68</v>
       </c>
       <c r="F106" s="6">
-        <f t="shared" si="1"/>
-        <v>37.4</v>
-      </c>
-      <c r="H106" s="23" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A107" s="13" t="s">
-        <v>17</v>
+        <v>7.96</v>
+      </c>
+      <c r="H106" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A107" s="14" t="s">
+        <v>276</v>
       </c>
       <c r="B107" s="26" t="s">
-        <v>244</v>
-      </c>
-      <c r="C107" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="D107" s="7">
-        <v>1</v>
-      </c>
-      <c r="E107" s="7">
-        <v>20.91</v>
+        <v>277</v>
+      </c>
+      <c r="C107" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D107" s="8">
+        <v>1</v>
+      </c>
+      <c r="E107" s="8">
+        <v>28.78</v>
       </c>
       <c r="F107" s="6">
-        <f t="shared" si="1"/>
-        <v>20.91</v>
-      </c>
-      <c r="H107" s="22" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+        <f t="shared" ref="F107:F109" si="3">D107*E107</f>
+        <v>28.78</v>
+      </c>
+      <c r="H107" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" s="14" t="s">
-        <v>61</v>
+        <v>280</v>
       </c>
       <c r="B108" s="26" t="s">
-        <v>251</v>
-      </c>
-      <c r="C108" s="11" t="s">
-        <v>74</v>
+        <v>283</v>
+      </c>
+      <c r="C108" s="10" t="s">
+        <v>282</v>
       </c>
       <c r="D108" s="8">
         <v>1</v>
       </c>
       <c r="E108" s="8">
-        <v>79.099999999999994</v>
+        <v>146.18</v>
       </c>
       <c r="F108" s="6">
-        <f t="shared" si="1"/>
-        <v>79.099999999999994</v>
-      </c>
-      <c r="H108" s="23" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A109" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B109" s="26" t="s">
-        <v>246</v>
-      </c>
-      <c r="C109" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="D109" s="7">
-        <v>1</v>
-      </c>
-      <c r="E109" s="7">
-        <v>16.260000000000002</v>
-      </c>
-      <c r="F109" s="6">
-        <f t="shared" si="1"/>
-        <v>16.260000000000002</v>
-      </c>
-      <c r="H109" s="22" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A110" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="B110" s="26" t="s">
-        <v>254</v>
-      </c>
-      <c r="C110" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="D110" s="28">
-        <v>1</v>
-      </c>
-      <c r="E110" s="28">
-        <v>5.35</v>
-      </c>
-      <c r="F110" s="6">
-        <f>D110*E110</f>
-        <v>5.35</v>
-      </c>
-      <c r="H110" s="1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A111" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="B111" s="26" t="s">
-        <v>256</v>
-      </c>
-      <c r="C111" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="D111" s="28">
-        <v>1</v>
-      </c>
-      <c r="E111" s="28">
-        <v>10.75</v>
-      </c>
-      <c r="F111" s="6">
-        <f>D111*E111</f>
-        <v>10.75</v>
-      </c>
-      <c r="H111" s="1" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A112" s="27" t="s">
-        <v>260</v>
-      </c>
-      <c r="B112" s="26" t="s">
-        <v>263</v>
-      </c>
-      <c r="C112" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="D112" s="28">
-        <v>1</v>
-      </c>
-      <c r="E112" s="28">
-        <v>6.68</v>
-      </c>
-      <c r="F112" s="6">
-        <v>7.96</v>
-      </c>
-      <c r="H112" s="1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A113" s="14" t="s">
-        <v>276</v>
-      </c>
-      <c r="B113" s="26" t="s">
-        <v>277</v>
-      </c>
-      <c r="C113" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="D113" s="8">
-        <v>1</v>
-      </c>
-      <c r="E113" s="8">
-        <v>28.78</v>
-      </c>
-      <c r="F113" s="6">
-        <f t="shared" ref="F113:F115" si="3">D113*E113</f>
-        <v>28.78</v>
-      </c>
-      <c r="H113" s="1" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A114" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="B114" s="26" t="s">
-        <v>283</v>
-      </c>
-      <c r="C114" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="D114" s="8">
-        <v>1</v>
-      </c>
-      <c r="E114" s="8">
-        <v>146.18</v>
-      </c>
-      <c r="F114" s="6">
         <f t="shared" si="3"/>
         <v>146.18</v>
       </c>
-      <c r="H114" s="1" t="s">
+      <c r="H108" s="1" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A115" s="14" t="s">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A109" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="B115" s="26" t="s">
+      <c r="B109" s="26" t="s">
         <v>284</v>
       </c>
-      <c r="C115" s="10" t="s">
+      <c r="C109" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="D115" s="8">
-        <v>1</v>
-      </c>
-      <c r="E115" s="8">
+      <c r="D109" s="8">
+        <v>1</v>
+      </c>
+      <c r="E109" s="8">
         <v>36.06</v>
       </c>
-      <c r="F115" s="6">
+      <c r="F109" s="6">
         <f t="shared" si="3"/>
         <v>36.06</v>
       </c>
-      <c r="H115" s="30" t="s">
+      <c r="H109" s="30" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="116" spans="1:11" s="36" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A116" s="31" t="s">
+    <row r="110" spans="1:11" s="36" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A110" s="31" t="s">
         <v>288</v>
       </c>
-      <c r="B116" s="32" t="s">
+      <c r="B110" s="32" t="s">
         <v>289</v>
       </c>
-      <c r="C116" s="33" t="s">
+      <c r="C110" s="33" t="s">
         <v>290</v>
       </c>
-      <c r="D116" s="34">
+      <c r="D110" s="34">
         <v>2</v>
       </c>
-      <c r="E116" s="34">
+      <c r="E110" s="34">
         <v>7.82</v>
       </c>
-      <c r="F116" s="35">
-        <f t="shared" ref="F116:F122" si="4">D116*E116</f>
+      <c r="F110" s="35">
+        <f t="shared" ref="F110:F116" si="4">D110*E110</f>
         <v>15.64</v>
       </c>
-      <c r="H116" s="37" t="s">
+      <c r="H110" s="37" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="117" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A117" s="38" t="s">
+    <row r="111" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A111" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B117" s="43" t="s">
+      <c r="B111" s="43" t="s">
         <v>292</v>
       </c>
-      <c r="C117" s="44" t="s">
+      <c r="C111" s="44" t="s">
         <v>293</v>
       </c>
-      <c r="D117" s="39">
+      <c r="D111" s="39">
         <v>2</v>
       </c>
-      <c r="E117" s="39">
+      <c r="E111" s="39">
         <v>14.99</v>
       </c>
-      <c r="F117" s="40">
+      <c r="F111" s="40">
         <f t="shared" si="4"/>
         <v>29.98</v>
       </c>
-      <c r="G117" s="41"/>
-      <c r="H117" s="42" t="s">
+      <c r="G111" s="41"/>
+      <c r="H111" s="42" t="s">
         <v>294</v>
       </c>
-      <c r="I117" s="41"/>
-      <c r="J117" s="41"/>
-      <c r="K117" s="41"/>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A118" s="14"/>
-      <c r="B118" s="26"/>
-      <c r="C118" s="10"/>
-      <c r="D118" s="8"/>
-      <c r="E118" s="8"/>
-      <c r="F118" s="6">
+      <c r="I111" s="41"/>
+      <c r="J111" s="41"/>
+      <c r="K111" s="41"/>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A112" s="14"/>
+      <c r="B112" s="26"/>
+      <c r="C112" s="10"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="6">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H118" s="10"/>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A119" s="14"/>
-      <c r="B119" s="26"/>
-      <c r="C119" s="10"/>
-      <c r="D119" s="8"/>
-      <c r="E119" s="8"/>
-      <c r="F119" s="6">
+      <c r="H112" s="10"/>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A113" s="14"/>
+      <c r="B113" s="26"/>
+      <c r="C113" s="10"/>
+      <c r="D113" s="8"/>
+      <c r="E113" s="8"/>
+      <c r="F113" s="6">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H119" s="10"/>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A120" s="14"/>
-      <c r="B120" s="26"/>
-      <c r="C120" s="10"/>
-      <c r="D120" s="8"/>
-      <c r="E120" s="8"/>
-      <c r="F120" s="6">
+      <c r="H113" s="10"/>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A114" s="14"/>
+      <c r="B114" s="26"/>
+      <c r="C114" s="10"/>
+      <c r="D114" s="8"/>
+      <c r="E114" s="8"/>
+      <c r="F114" s="6">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H120" s="10"/>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A121" s="14"/>
-      <c r="B121" s="26"/>
-      <c r="C121" s="10"/>
-      <c r="D121" s="8"/>
-      <c r="E121" s="8"/>
-      <c r="F121" s="6">
+      <c r="H114" s="10"/>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A115" s="14"/>
+      <c r="B115" s="26"/>
+      <c r="C115" s="10"/>
+      <c r="D115" s="8"/>
+      <c r="E115" s="8"/>
+      <c r="F115" s="6">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H121" s="10"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A122" s="27"/>
-      <c r="B122" s="26"/>
-      <c r="C122" s="10"/>
-      <c r="D122" s="28"/>
-      <c r="E122" s="28"/>
-      <c r="F122" s="6">
+      <c r="H115" s="10"/>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A116" s="27"/>
+      <c r="B116" s="26"/>
+      <c r="C116" s="10"/>
+      <c r="D116" s="28"/>
+      <c r="E116" s="28"/>
+      <c r="F116" s="6">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H122" s="10"/>
+      <c r="H116" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -4632,22 +4560,22 @@
     <hyperlink ref="H89" r:id="rId86" display="https://www.grainger.com/product/1VFX8?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=6d4e1d7881c4014dc580a65ce33a0287e6d4e842f558a81fadd5dcde7a752909&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{460DB0C6-014B-408D-A50E-7C7CB6F31C51}"/>
     <hyperlink ref="H90" r:id="rId87" display="https://www.dwyeromega.com/en-us/oem-style-compact-pressure-transmitters/PX119/p/PX159A-060G5V" xr:uid="{B046FF95-BF93-46C9-B8CE-FB723F36F53A}"/>
     <hyperlink ref="H91" r:id="rId88" display="https://www.grainger.com/product/Hex-Tap-Bolt-Stainless-Steel-41UH04?gucid=n:n:em:owned:wwg:deliveryConfirmation:apz_1&amp;emcid=body:pdpurl" xr:uid="{5ACA225F-14EA-4C12-8992-27C2A205D0A2}"/>
-    <hyperlink ref="H105" r:id="rId89" xr:uid="{66B68E33-6FB6-4B9E-8DEE-AD4543BA3948}"/>
-    <hyperlink ref="H104" r:id="rId90" display="https://www.dwyeromega.com/en-us/oem-style-compact-pressure-transmitters/PX119/p/PX159A-060G5V" xr:uid="{E0383BBC-B224-42C5-8E0D-F57DE49C5FA3}"/>
-    <hyperlink ref="H106" r:id="rId91" xr:uid="{A3D63FAB-C850-40A1-A637-DF41091272C8}"/>
-    <hyperlink ref="H107" r:id="rId92" display="https://www.grainger.com/product/20XM58?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=5fbed57f928e0d20c3753de78a2b9a38ffd20234e126526a2f6d6b4fe4e772db&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{2C07356E-8DE4-40F2-A1AD-4E8492786388}"/>
-    <hyperlink ref="H108" r:id="rId93" xr:uid="{94CC04D7-EB9A-450B-BB5C-C756BC4DE898}"/>
-    <hyperlink ref="H109" r:id="rId94" display="https://www.grainger.com/product/IGUS-Flanged-Sleeve-Bearing-Polymer-2NCK6" xr:uid="{83384CCF-7FBA-4E7B-9A1D-1C877A885273}"/>
-    <hyperlink ref="H110" r:id="rId95" display="https://www.grainger.com/product/Hex-Nut-Std-Hex-2FE69" xr:uid="{85183601-0793-4417-9C08-9D53A5FEB9B5}"/>
-    <hyperlink ref="H111" r:id="rId96" display="https://www.grainger.com/product/Mil-Spec-Flat-Washer-18-8-2DNV3" xr:uid="{FC3AB918-B994-4AB5-AFC0-90ECDBC2A4C8}"/>
-    <hyperlink ref="H112" r:id="rId97" xr:uid="{FDEFAFD3-3687-4641-964A-8BC9B3E42512}"/>
+    <hyperlink ref="H99" r:id="rId89" xr:uid="{66B68E33-6FB6-4B9E-8DEE-AD4543BA3948}"/>
+    <hyperlink ref="H98" r:id="rId90" display="https://www.dwyeromega.com/en-us/oem-style-compact-pressure-transmitters/PX119/p/PX159A-060G5V" xr:uid="{E0383BBC-B224-42C5-8E0D-F57DE49C5FA3}"/>
+    <hyperlink ref="H100" r:id="rId91" xr:uid="{A3D63FAB-C850-40A1-A637-DF41091272C8}"/>
+    <hyperlink ref="H101" r:id="rId92" display="https://www.grainger.com/product/20XM58?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=5fbed57f928e0d20c3753de78a2b9a38ffd20234e126526a2f6d6b4fe4e772db&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{2C07356E-8DE4-40F2-A1AD-4E8492786388}"/>
+    <hyperlink ref="H102" r:id="rId93" xr:uid="{94CC04D7-EB9A-450B-BB5C-C756BC4DE898}"/>
+    <hyperlink ref="H103" r:id="rId94" display="https://www.grainger.com/product/IGUS-Flanged-Sleeve-Bearing-Polymer-2NCK6" xr:uid="{83384CCF-7FBA-4E7B-9A1D-1C877A885273}"/>
+    <hyperlink ref="H104" r:id="rId95" display="https://www.grainger.com/product/Hex-Nut-Std-Hex-2FE69" xr:uid="{85183601-0793-4417-9C08-9D53A5FEB9B5}"/>
+    <hyperlink ref="H105" r:id="rId96" display="https://www.grainger.com/product/Mil-Spec-Flat-Washer-18-8-2DNV3" xr:uid="{FC3AB918-B994-4AB5-AFC0-90ECDBC2A4C8}"/>
+    <hyperlink ref="H106" r:id="rId97" xr:uid="{FDEFAFD3-3687-4641-964A-8BC9B3E42512}"/>
     <hyperlink ref="H95" r:id="rId98" xr:uid="{29622D1D-FB83-4317-A033-D7DD9D94A271}"/>
     <hyperlink ref="H94" r:id="rId99" xr:uid="{5FC8DB1C-6249-4551-B238-6394EA039EB9}"/>
-    <hyperlink ref="H113" r:id="rId100" display="https://www.grainger.com/product/BANJO-Inline-Strainer-Polypropylene-3ELX2" xr:uid="{5DDCF04D-0B2B-4400-9BF3-CBBD33627CF9}"/>
-    <hyperlink ref="H114" r:id="rId101" display="https://www.grainger.com/product/BELL-GOSSETT-Water-Pressure-Reducing-Valve-6LFA3" xr:uid="{704D45CE-3BF8-44FB-A2F9-FBD42F90D381}"/>
-    <hyperlink ref="H115" r:id="rId102" xr:uid="{DA2A078E-95DA-4F11-A662-702B09E6F14A}"/>
-    <hyperlink ref="H116" r:id="rId103" display="https://www.grainger.com/product/803H45?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=a98025ace82cfe3e9959eb0e2dd5f9501b4a446af591eb4540e15aea507809d7&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{05215C5A-3A93-40D1-9E83-5B1ABEB0BD2B}"/>
-    <hyperlink ref="H117" r:id="rId104" display="https://www.grainger.com/product/20KF99?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=a98025ace82cfe3e9959eb0e2dd5f9501b4a446af591eb4540e15aea507809d7&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{0F353E44-E7EA-4190-9112-90CB38990103}"/>
+    <hyperlink ref="H107" r:id="rId100" display="https://www.grainger.com/product/BANJO-Inline-Strainer-Polypropylene-3ELX2" xr:uid="{5DDCF04D-0B2B-4400-9BF3-CBBD33627CF9}"/>
+    <hyperlink ref="H108" r:id="rId101" display="https://www.grainger.com/product/BELL-GOSSETT-Water-Pressure-Reducing-Valve-6LFA3" xr:uid="{704D45CE-3BF8-44FB-A2F9-FBD42F90D381}"/>
+    <hyperlink ref="H109" r:id="rId102" xr:uid="{DA2A078E-95DA-4F11-A662-702B09E6F14A}"/>
+    <hyperlink ref="H110" r:id="rId103" display="https://www.grainger.com/product/803H45?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=a98025ace82cfe3e9959eb0e2dd5f9501b4a446af591eb4540e15aea507809d7&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{05215C5A-3A93-40D1-9E83-5B1ABEB0BD2B}"/>
+    <hyperlink ref="H111" r:id="rId104" display="https://www.grainger.com/product/20KF99?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=a98025ace82cfe3e9959eb0e2dd5f9501b4a446af591eb4540e15aea507809d7&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{0F353E44-E7EA-4190-9112-90CB38990103}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId105"/>

</xml_diff>